<commit_message>
Add household/home sleep environment papers to first tab
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017saKLUxckuv8JPxf8F2UXy
</commit_message>
<xml_diff>
--- a/sleep_literature_review.xlsx
+++ b/sleep_literature_review.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,9 +45,15 @@
     </font>
     <font>
       <b val="1"/>
+      <i val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +63,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -100,13 +111,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -474,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -680,9 +695,264 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Household / home sleep environment (bed-sharing &amp; room-sharing, crowding, housing type/quality, neighborhood physical environment)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="118" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ijerph192013599</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Development and Initial Validation of the Assessment of Sleep Environment (ASE)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Grandner et al., 2022, Int J Environ Res Public Health 19(20):13599</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>US; 1,007 adults 22-60 (SHADES study)</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>13-item validated self-report scale of the subjective bedroom environment (light, temperature, safety, noise, comfort, humidity, smell); the physical-environment score is associated with insomnia symptoms and sleep quality. The most directly relevant validated instrument for the physical home sleep environment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="118" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/25386692/</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Sleep and the Housing and Neighborhood Environment of Urban Latino Adults Living in Low-Income Housing: The AHOME Study</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Chambers, Pichardo &amp; Rosenbaum, 2016, Behavioral Sleep Medicine</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>US; 371 low-income urban Latino adults, Bronx NY</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Operationalizes household crowding (persons per room) plus perceived building problems; crowding was associated with reduced odds of long sleep, and neighborhood disorder / building problems with more sleep disturbance and poorer quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="118" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/29561769/</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Black-White Differences in Housing Type and Sleep Duration as Well as Sleep Difficulties in the United States</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Johnson, Thorpe, McGrath, Jackson &amp; Jackson, 2018, Int J Environ Res Public Health 15(4):564</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>US; 226,208 adults (NHIS 2004-2015)</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Housing type (mobile home/trailer vs house/apartment) is linked to worse sleep; documents housing as a driver of Black-White sleep disparities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="118" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s11524-019-00418-5</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Broken Windows, Broken Zzs: Poor Housing and Neighborhood Conditions Are Associated with Objective Measures of Sleep Health</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Troxel et al., 2020, Journal of Urban Health</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>US; low-income adults, Pittsburgh PA (actigraphy)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Combined interior/exterior housing-problem measure (pests, broken windows); adverse housing conditions were independently associated with shorter actigraphic total sleep time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="118" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC8844874/</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Exterior Housing Conditions Are Associated With Objective Measures of Poor Sleep</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Okoye, Perrin, Szanton &amp; Spira, 2021, Sleep Health</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>US; 136 low-income, predominantly African-American older adults with disabilities</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Uses third-party-rated inside/outside home and neighborhood disrepair; &gt;=1 outside-home disrepair condition was associated with ~36 min shorter total sleep time, more WASO, and lower sleep efficiency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="118" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1093/aje/kwad016</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Neighborhood Built Environment and Sleep Health: A Longitudinal Study in Low-Income and Predominantly African-American Neighborhoods</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Kim et al., 2023, American Journal of Epidemiology 192(5):736-747</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>US; 1,051 residents, Pittsburgh (PHRESH Zzz, 2013-2018)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Longitudinal repeated measures of the neighborhood physical/built environment linked to objective sleep outcomes in disadvantaged neighborhoods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="118" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/23161266/</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Association Between Housing Quality and Sleep Quality Among Latino Farmworkers</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Sandberg et al., 2014, Journal of Immigrant and Minority Health</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>US; 371 male Latino farmworkers, North Carolina</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Uses a housing-quality inventory (including air conditioning); access to air conditioning was positively and independently associated with good sleep quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="118" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/abs/pii/S0277953625008548</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Housing crowding and sleep health in urban China (psychosocial mediation)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>2025, Social Science &amp; Medicine (author byline not confirmed from snippets)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>China; nationally representative adults (2022 China Family Panel Studies)</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Housing crowding was associated with abnormal sleep duration, partially mediated by subjective well-being and self-perceived social status. Verify exact title &amp; authors on the publisher page before citing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="118" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/cdev.13146</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Parent-Infant Room Sharing During the First Months of Life</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Beijers, Cassidy, Lustermans &amp; de Weerth, 2019, Child Development 90(4):1350-1367</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Netherlands; 193 infant-parent dyads (daily diary, followed to age 6-8)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Measures room-sharing via a daily infant sleep-location diary over the first 6 months; more weeks of room sharing was linked to higher maternal-rated sleep quality and prosocial behavior, with no adverse effects.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
@@ -691,6 +961,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1393,86 +1672,86 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Verification &amp; scope notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr"/>
+      <c r="A2" s="8" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>All 24 papers were verified: every DOI / PubMed ID / URL resolves to the stated article, and titles, authors, journals, and years match.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Peer-reviewed journal articles only. US and/or Latino/Hispanic populations prioritized; non-US or non-Latino items are foundational instruments/methods and are flagged in the Population column.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr"/>
+      <c r="A5" s="8" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Caveats:</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>- Community Interventions row 4 (Dominican Republic, Sleep Health 2016) and row 6 (Nuestro Sueno protocol, Sleep Medicine 2026): the articles definitely exist at the given URLs with confirmed titles, but author bylines could not be independently confirmed from search snippets. Verify authors on the publisher page.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>- Nuestro Sueno is a study PROTOCOL - it reports no outcome results yet.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>- ICC row 6 (Inhulsen 2022) reports an ASSUMED school-level ICC of 0.10 used in a power calculation, not an empirically estimated value.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr"/>
+      <c r="A10" s="8" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Literature gaps identified:</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>- No widely validated standalone 'family sleep health scale' beyond the FISH.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>- No completed, peer-reviewed promotora-delivered sleep intervention in US Latino adults with reported sleep outcomes yet (niche is at protocol/pilot stage).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>- Empirically estimated household- or clinic-level clustering ICCs for sleep are scarce; the twin heritability (0.31) and the assumed school-level ICC (0.10) are the closest anchors for multilevel design planning.</t>
         </is>

</xml_diff>

<commit_message>
Restructure: Tab 1 scored sleep instruments, new Tab 2 family-level sleep factors
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017saKLUxckuv8JPxf8F2UXy
</commit_message>
<xml_diff>
--- a/sleep_literature_review.xlsx
+++ b/sleep_literature_review.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Family Sleep Measures" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Community Sleep Interventions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Family Cohesion Measures" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ICC Findings in Sleep Research" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Notes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sleep Instruments (scored)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Family Factors &amp; Sleep" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Community Interventions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Family Cohesion Measures" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ICC in Sleep Research" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Notes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,7 +490,347 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="64" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TAB 1 - Sleep Instruments: scored household/family/environment measures (MOST USEFUL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Paper link</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Instrument / Title</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Authors / Year / Journal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>What it scores + structure / validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="128" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ijerph192013599</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Assessment of Sleep Environment (ASE) - Development and Initial Validation</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Grandner et al., 2022, Int J Environ Res Public Health 19(20):13599</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>US; 1,007 adults 22-60 (SHADES)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>STAR INSTRUMENT for the home sleep environment. 13-item validated self-report scale scoring the subjective bedroom environment (light, temperature, safety, noise, comfort, humidity, smell). Higher score = more disruptive environment; associated with insomnia symptoms and poorer sleep quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="128" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/0883073808321044</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Family Inventory of Sleep Habits (FISH)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Malow et al., 2009, J Child Neurol 24(1):19-24</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>US; children 4-10 yr (ASD + typically developing)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Parent-report FAMILY-level sleep-hygiene score: daytime habits, pre-bedtime routine, bedtime routine, sleep environment, and parental bedtime behaviors summed into a sleep-hygiene score. Reported valid and reliable; the most established family-level scored sleep instrument.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="128" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5664/jcsm.10110</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Children's and Adolescents' Sleep Environment Scale (CASES)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Peltz, Rogge, Elmore-Staton, Spilsbury &amp; Buckhalt, 2022, J Clin Sleep Med 18(10):2353-2365</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>US; 840 caregivers, children 5-18 yr</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>13-item parent-report scale scoring the child's sleep environment across 3 factors: general environmental hazards, bedding availability, and presence of electronics. Validated via EFA/CFA in split-half samples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="128" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10862-009-9143-3</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Bedtime Routines Questionnaire (BRQ)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Henderson &amp; Jordan, 2010, J Psychopathol Behav Assess 32(2):271-280</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>US; 226 caregivers of children 2-8 yr</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>31-item parent-report score of children's bedtime routines (reactive vs. consistent routines). Solid factor structure, adequate internal consistency, fair validity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="128" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jsr.12059</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Adolescent Sleep Hygiene Scale - Revised (ASHS-r)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Storfer-Isser, LeBourgeois, Harsh, Tompsett &amp; Redline, 2013, J Sleep Res 22(6)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>US; urban adolescents 16-19</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Self-report sleep-hygiene score; CFA yielded 6 factors INCLUDING a scored 'sleep environment' subscale (plus physiological, behavioral-arousal, cognitive/emotional, daytime sleep, sleep stability). Higher = better hygiene; total associated with sleep duration/efficiency and daytime sleepiness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="128" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/1359105309346342</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Sleep Hygiene Practice Scale (SHPS)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Yang, Lin, Hsu &amp; Cheng, 2010, J Health Psychol 15(1):147-155</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Taiwan; adults (good sleepers + insomnia patients)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>30 items, 6-point Likert, total 30-180, across 4 domains INCLUDING a scored 'sleep environment' domain (plus schedule/timing, arousal behaviors, eating/drinking). Higher = more maladaptive; environment domain correlated with PSQI sleep quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="128" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.5664/jcsm.2486</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Children's Report of Sleep Patterns (CRSP)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Meltzer, Avis, Biggs, Reynolds, Crabtree &amp; Bevans, 2013, J Clin Sleep Med 9(3):235-245</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>US; children 8-12 (Denver)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Child self-report with 3 modules; the Sleep Hygiene module contains a scored 'environmental' sleep-hygiene subscale (with physiological, cognitive, emotional, routines, stability). Reliable/valid; modules usable independently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="128" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/15402002.2020.1714625</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Pediatric Sleep Practices Questionnaire (PSPQ)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Meltzer, Forrest, de la Motte, Mindell &amp; Bevans, 2021, Behav Sleep Med 19(1)</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>US; youth 8-17 (n=307)</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>15 items scoring 5 sleep practices INCLUDING a scored 'sleep environment' (room environment) subscale (plus timing, routines/consistency, technology use, parental presence). Subscale scores summed; CFA-supported, clinically valid vs. parent-identified sleep problems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="128" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.pedn.2017.02.033</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Parent Newborn Sleep Safety Survey</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Whiteside-Mansell, Nabaweesi, Caballero, Mullins, Miller &amp; Aitken, 2017, J Pediatr Nurs 35:30-35</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>US; parents of newborns, high-risk families (n=72)</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>14 items (mostly 4-point frequency) scoring parent adherence to AAP safe-sleep-ENVIRONMENT recommendations (position, surface, bedding, location). Validated against direct observation (item Kappas fair-to-excellent) as a scored alternative to observation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="128" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10902-020-00302-z</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Household Crowding Index (persons-per-room / bedroom-standard) - methodological validation</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Torshizian &amp; Grimes, 2021, J Happiness Stud 22:1925-1951 (also Cable &amp; Sacker, 2019, SSM-Population Health 8:100439, https://doi.org/10.1016/j.ssmph.2019.100439)</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Household-level; NZ and UK samples</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>A COMPUTED household index = persons / rooms (or Canadian / Bedroom Standard variants). These two peer-reviewed studies compare and validate the objective crowding measures against socioeconomic/health/wellbeing outcomes - the citable methodological basis for a persons-per-room household sleep-environment index.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId10"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -502,7 +843,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>1. Family Sleep Measures</t>
+          <t>TAB 2 - Family / household-level factors associated with sleep</t>
         </is>
       </c>
     </row>
@@ -533,234 +874,202 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="118" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1177/0883073808321044</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>A sleep habits questionnaire for children with autism spectrum disorders (introduces the Family Inventory of Sleep Habits, FISH)</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Malow et al., 2009, J Child Neurol 24(1):19-24</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>US; children 4-10 yr, ASD + typically developing</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>FISH is a parent-report measure of family/child sleep hygiene (daytime habits, pre-bedtime, bedtime routine, sleep environment, parental bedtime behaviors); reported valid and reliable in ASD. The most established family-level sleep instrument.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="118" customHeight="1">
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Family routines, parenting &amp; sociodemographics</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="128" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s10862-009-9143-3</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/36055935/</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Development and Preliminary Evaluation of the Bedtime Routines Questionnaire (BRQ)</t>
+          <t>Sleep health among U.S. Hispanic/Latinx children: An examination of correlates of meeting sleep duration recommendations</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Henderson &amp; Jordan, 2010, J Psychopathol Behav Assess 32(2):271-280</t>
+          <t>Schmied et al., 2022, Sleep Health</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>US; 226 caregivers of children 2-8 yr</t>
+          <t>US, Hispanic/Latinx; 1,165 children (~6.4 yr)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>31-item parent-report measure of children's bedtime routines; solid factor structure, adequate internal consistency, fair validity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="118" customHeight="1">
+          <t>61.4% met sleep-duration guidelines; a regular/consistent bedtime and living above the poverty threshold significantly raised odds of meeting recommendations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="128" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.5664/jcsm.10110</t>
+          <t>https://doi.org/10.1016/j.sleh.2021.11.004</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>The development of a scale to assess children's and adolescents' sleep environments</t>
+          <t>Sleep-related parenting self-efficacy and parent-reported sleep in young children: A dyadic analysis of parental actor and partner effects</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Peltz, Rogge, Elmore-Staton, Spilsbury &amp; Buckhalt, 2022, J Clin Sleep Med 18(10):2353-2365</t>
+          <t>Werner, Mayer &amp; Lohaus, 2022, Sleep Health 8(1):54-61</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>US; 840 caregivers, children 5-18 yr</t>
+          <t>Germany; 131 mother-father dyads</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>13-item parent-report scale with 3 factors (environmental hazards, bedding availability, presence of electronics); validated via EFA/CFA in split-half samples.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="118" customHeight="1">
+          <t>Actor-partner interdependence model linking sleep-related parenting self-efficacy to child sleep problems; demonstrates dyadic (mother/father) family-level effects on child sleep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="128" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.sleh.2021.11.004</t>
+          <t>https://doi.org/10.1097/MOP.0000000000001306</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Sleep-related parenting self-efficacy and parent-reported sleep in young children: A dyadic analysis of parental actor and partner effects</t>
+          <t>Assessing sleep behaviors in Latino children and adolescents: what is known, what are we missing, and how do we move forward?</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Werner, Mayer &amp; Lohaus, 2022, Sleep Health 8(1):54-61</t>
+          <t>Blanco, Hyde &amp; Martinez, 2024, Curr Opin Pediatr 36(1):17-22</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Germany (non-US); 131 mother-father dyads</t>
+          <t>US, Latino (review)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Actor-partner interdependence model measuring sleep-related parenting self-efficacy dyadically; links parental self-efficacy to child sleep problems. Included as a dyadic-measurement exemplar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="118" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/36055935/</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Sleep health among U.S. Hispanic/Latinx children: An examination of correlates of meeting sleep duration recommendations</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Schmied et al., 2022, Sleep Health</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>US, Hispanic/Latinx; 1,165 children (mean ~6.4 yr)</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>61.4% met sleep-duration guidelines; a regular/consistent bedtime and living above the poverty threshold significantly raised odds of meeting recommendations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="118" customHeight="1">
+          <t>Review arguing that cultural/contextual family factors (co-sleeping, bed-sharing) must be accounted for when measuring Latino family sleep - a measurement-gap analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Household crowding &amp; room/bed sharing</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="128" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1097/MOP.0000000000001306</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/25386692/</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Assessing sleep behaviors in Latino children and adolescents: what is known, what are we missing, and how do we move forward?</t>
+          <t>Sleep and the Housing and Neighborhood Environment of Urban Latino Adults Living in Low-Income Housing: The AHOME Study</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Blanco, Hyde &amp; Martinez, 2024, Curr Opin Pediatr 36(1):17-22</t>
+          <t>Chambers, Pichardo &amp; Rosenbaum, 2016, Behav Sleep Med</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>US, Latino (review)</t>
+          <t>US, Latino; 371 low-income adults, Bronx NY</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Identifies the need to account for cultural/contextual family factors (co-sleeping, bed-sharing) in sleep measurement; a measurement-gap analysis relevant to family sleep instruments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Household / home sleep environment (bed-sharing &amp; room-sharing, crowding, housing type/quality, neighborhood physical environment)</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="118" customHeight="1">
+          <t>Household crowding (persons/room) was associated with reduced odds of long sleep; neighborhood disorder and perceived building problems tied to more sleep disturbance / poorer quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="128" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/abs/pii/S0277953625008548</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Housing crowding and sleep health in urban China (psychosocial mediation)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>2025, Social Science &amp; Medicine (author byline not confirmed from snippets)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>China; nationally representative adults (CFPS 2022)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Housing crowding associated with abnormal sleep duration, partially mediated by subjective well-being and self-perceived social status. Verify exact title/authors before citing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="128" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/ijerph192013599</t>
+          <t>https://doi.org/10.1111/cdev.13146</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Development and Initial Validation of the Assessment of Sleep Environment (ASE)</t>
+          <t>Parent-Infant Room Sharing During the First Months of Life</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Grandner et al., 2022, Int J Environ Res Public Health 19(20):13599</t>
+          <t>Beijers, Cassidy, Lustermans &amp; de Weerth, 2019, Child Development 90(4):1350-1367</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>US; 1,007 adults 22-60 (SHADES study)</t>
+          <t>Netherlands; 193 infant-parent dyads</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>13-item validated self-report scale of the subjective bedroom environment (light, temperature, safety, noise, comfort, humidity, smell); the physical-environment score is associated with insomnia symptoms and sleep quality. The most directly relevant validated instrument for the physical home sleep environment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="118" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/25386692/</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Sleep and the Housing and Neighborhood Environment of Urban Latino Adults Living in Low-Income Housing: The AHOME Study</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Chambers, Pichardo &amp; Rosenbaum, 2016, Behavioral Sleep Medicine</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>US; 371 low-income urban Latino adults, Bronx NY</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Operationalizes household crowding (persons per room) plus perceived building problems; crowding was associated with reduced odds of long sleep, and neighborhood disorder / building problems with more sleep disturbance and poorer quality.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="118" customHeight="1">
+          <t>More weeks of room sharing (daily sleep-location diary) linked to higher maternal-rated sleep quality and prosocial behavior, with no adverse effects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Housing type / quality &amp; neighborhood physical environment</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+    </row>
+    <row r="12" ht="128" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/29561769/</t>
@@ -783,11 +1092,11 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Housing type (mobile home/trailer vs house/apartment) is linked to worse sleep; documents housing as a driver of Black-White sleep disparities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="118" customHeight="1">
+          <t>Housing type (mobile home/trailer vs house/apartment) linked to worse sleep; documents housing as a driver of Black-White sleep disparities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="128" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s11524-019-00418-5</t>
@@ -805,16 +1114,16 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>US; low-income adults, Pittsburgh PA (actigraphy)</t>
+          <t>US; low-income adults, Pittsburgh (actigraphy)</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Combined interior/exterior housing-problem measure (pests, broken windows); adverse housing conditions were independently associated with shorter actigraphic total sleep time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="118" customHeight="1">
+          <t>Combined interior/exterior housing-problem measure; adverse housing conditions independently associated with shorter actigraphic total sleep time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="128" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC8844874/</t>
@@ -832,16 +1141,16 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>US; 136 low-income, predominantly African-American older adults with disabilities</t>
+          <t>US; 136 low-income, predominantly African-American older adults</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Uses third-party-rated inside/outside home and neighborhood disrepair; &gt;=1 outside-home disrepair condition was associated with ~36 min shorter total sleep time, more WASO, and lower sleep efficiency.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="118" customHeight="1">
+          <t>&gt;=1 outside-home disrepair condition (third-party-rated) associated with ~36 min shorter total sleep time, more WASO, and lower sleep efficiency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="128" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1093/aje/kwad016</t>
@@ -859,7 +1168,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>US; 1,051 residents, Pittsburgh (PHRESH Zzz, 2013-2018)</t>
+          <t>US; 1,051 residents, Pittsburgh (PHRESH Zzz)</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -868,7 +1177,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="118" customHeight="1">
+    <row r="16" ht="128" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>https://pubmed.ncbi.nlm.nih.gov/23161266/</t>
@@ -886,318 +1195,34 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>US; 371 male Latino farmworkers, North Carolina</t>
+          <t>US, Latino; 371 male farmworkers, NC</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Uses a housing-quality inventory (including air conditioning); access to air conditioning was positively and independently associated with good sleep quality.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="118" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sciencedirect.com/science/article/abs/pii/S0277953625008548</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Housing crowding and sleep health in urban China (psychosocial mediation)</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>2025, Social Science &amp; Medicine (author byline not confirmed from snippets)</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>China; nationally representative adults (2022 China Family Panel Studies)</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Housing crowding was associated with abnormal sleep duration, partially mediated by subjective well-being and self-perceived social status. Verify exact title &amp; authors on the publisher page before citing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="118" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1111/cdev.13146</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Parent-Infant Room Sharing During the First Months of Life</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Beijers, Cassidy, Lustermans &amp; de Weerth, 2019, Child Development 90(4):1350-1367</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Netherlands; 193 infant-parent dyads (daily diary, followed to age 6-8)</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>Measures room-sharing via a daily infant sleep-location diary over the first 6 months; more weeks of room sharing was linked to higher maternal-rated sleep quality and prosocial behavior, with no adverse effects.</t>
+          <t>Housing-quality inventory (incl. air conditioning); access to air conditioning positively and independently associated with good sleep quality.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
+    <mergeCell ref="A11:E11"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>2. Community Sleep Interventions</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Paper link</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Authors / Year / Journal</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Key relevant finding(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="118" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1177/00099228231207307</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>A Pilot Randomized Control Trial Demonstrating the Efficacy of the SIESTA Sleep Hygiene Intervention</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Koinis-Mitchell et al., 2024, Clinical Pediatrics 63(8):1062-1077</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>US + Latino; urban Latino middle-schoolers (Providence RI &amp; San Juan PR); school-based, bilingual</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Actigraphy sleep duration rose 13.3% (~45 min) in SIESTA vs 7.2% (~25 min) in controls; child- and caregiver-reported sleep disturbances significantly decreased through 4-month follow-up.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="118" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.5664/jcsm.8510</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Tailored Approach to Sleep Health Education (TASHE): a randomized controlled trial of a web-based application</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Jean-Louis et al., 2020, J Clin Sleep Med 16(8):1331-1341</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>US, Black; 194 adults at high OSA risk; community-engaged (barbershops, salons, places of worship)</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>TASHE group showed increased sleep hygiene over 6 months vs control; no significant change in OSA beliefs or knowledge.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="118" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1111/jsr.14213</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Effectiveness of peer-delivered sleep health education and social support in increasing OSA evaluation among at-risk blacks</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Jean-Louis et al., 2025, J Sleep Res 34(1):e14213</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>US, Black; 319 adults at OSA risk; peer/community-delivered</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Peer-based social support and psychosocial factors favorably related to OSA evaluation/adherence behavior vs standard information.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="118" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sciencedirect.com/science/article/abs/pii/S2352721816000188</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Efficacy of sleep education in a Dominican Republic neighborhood through training of community health promoters</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>2016, Sleep Health (author byline not confirmed from snippets)</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Dominican Republic (Latino, non-US); community members + 9 health promoters</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Promoters' sleep-disorder knowledge improved after a 4-hr training, but community members' knowledge did not significantly change after promoter-delivered education.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="118" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.ctcp.2020.101121</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>A sleep hygiene and yoga intervention conducted in affordable housing communities: pilot study results and lessons for a future trial</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Spadola et al., 2020, Complement Ther Clin Pract 39:101121</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>US; low-income, racially/ethnically diverse adults (~19% Hispanic/Latino); community-based</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Significant pre/post improvements: sleep duration 5.4-&gt;6.9 h/night (p&lt;0.01), sleep-related impairment, sleep disturbance, and sleep-hygiene behaviors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="118" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S1389945726002583</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Protocol for Nuestro Sueno: a randomized trial of a couples-based intervention to improve PAP adherence and sleep health among Hispanic patients beginning PAP and their partners</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>2026, Sleep Medicine (protocol; NCT06649929; author byline not confirmed from snippets)</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>US + Latino; Hispanic couples; CHW-delivered telehealth</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>PROTOCOL ONLY - no outcomes yet. Pilot RCT testing a culturally adapted, community-health-worker-delivered couples intervention vs information control for PAP adherence and both partners' sleep.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1222,7 +1247,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>3. Family Cohesion Measures</t>
+          <t>TAB 3 - Community sleep interventions</t>
         </is>
       </c>
     </row>
@@ -1253,165 +1278,165 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="118" customHeight="1">
+    <row r="3" ht="128" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/j.1752-0606.2009.00175.x</t>
+          <t>https://doi.org/10.1177/00099228231207307</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>FACES IV and the Circumplex Model: Validation Study</t>
+          <t>A Pilot Randomized Control Trial Demonstrating the Efficacy of the SIESTA Sleep Hygiene Intervention</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Olson, 2011, J Marital Fam Ther 37(1):64-80</t>
+          <t>Koinis-Mitchell et al., 2024, Clinical Pediatrics 63(8):1062-1077</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>US adults</t>
+          <t>US + Latino; urban Latino middle-schoolers (Providence RI &amp; San Juan PR); school-based, bilingual</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Core validation of FACES IV; six scales span the cohesion continuum (balanced, disengaged, enmeshed) and flexibility, with strong concurrent, construct, and discriminant validity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="118" customHeight="1">
+          <t>Actigraphy sleep duration rose 13.3% (~45 min) in SIESTA vs 7.2% (~25 min) in controls; child- and caregiver-reported sleep disturbances significantly decreased through 4-month follow-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="128" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/31853517/</t>
+          <t>https://doi.org/10.5664/jcsm.8510</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Measurement Properties of Sabogal's Familism Scale: Findings from the HCHS/SOL Sociocultural Ancillary Study</t>
+          <t>Tailored Approach to Sleep Health Education (TASHE): a randomized controlled trial of a web-based application</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Campos et al., 2019, J Latinx Psychol 7(4):257-272 (DOI 10.1037/lat0000126)</t>
+          <t>Jean-Louis et al., 2020, J Clin Sleep Med 16(8):1331-1341</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>US Hispanic/Latino; N=5,313</t>
+          <t>US, Black; 194 adults at high OSA risk; community-engaged (barbershops, salons, places of worship)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Sabogal's 3-factor model (obligations, support, family as referents) fit well and was invariant across English/Spanish; good convergent/discriminant validity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="118" customHeight="1">
+          <t>TASHE group showed increased sleep hygiene over 6 months vs control; no significant change in OSA beliefs or knowledge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="128" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/0739986303256912</t>
+          <t>https://doi.org/10.1111/jsr.14213</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>A New Familism Scale for Use with Latino Populations</t>
+          <t>Effectiveness of peer-delivered sleep health education and social support in increasing OSA evaluation among at-risk blacks</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Lugo Steidel &amp; Contreras, 2003, Hisp J Behav Sci 25(3):312-330</t>
+          <t>Jean-Louis et al., 2025, J Sleep Res 34(1):e14213</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>US Latino adults; N=124</t>
+          <t>US, Black; 319 adults at OSA risk; peer/community-delivered</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>18-item scale, 4 factors (Support, Interconnectedness, Honor, Subjugation of Self), explaining ~51% of variance; overall alpha = .83.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="118" customHeight="1">
+          <t>Peer-based social support and psychosocial factors favorably related to OSA evaluation/adherence behavior vs standard information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="128" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/0272431609338178</t>
+          <t>https://www.sciencedirect.com/science/article/abs/pii/S2352721816000188</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>The Mexican American Cultural Values Scale for Adolescents and Adults (MACVS)</t>
+          <t>Efficacy of sleep education in a Dominican Republic neighborhood through training of community health promoters</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Knight et al., 2010, J Early Adolesc 30(3):444-481</t>
+          <t>2016, Sleep Health (author byline not confirmed from snippets)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>US Mexican American adolescents &amp; parents</t>
+          <t>Dominican Republic (Latino, non-US); community members + 9 health promoters</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>50-item, 9-subscale measure with three Familism subscales (Support, Referent, Obligation); supported the higher-order structure, reliability, and construct validity. English/Spanish.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="118" customHeight="1">
+          <t>Promoters' sleep-disorder knowledge improved after a 4-hr training, but community members' knowledge did not significantly change after promoter-delivered education.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="128" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/0739986305281125</t>
+          <t>https://doi.org/10.1016/j.ctcp.2020.101121</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Factorial invariance of a pan-Hispanic familism scale</t>
+          <t>A sleep hygiene and yoga intervention conducted in affordable housing communities: pilot study results and lessons for a future trial</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Villarreal, Blozis &amp; Widaman, 2005, Hisp J Behav Sci 27(4):409-425</t>
+          <t>Spadola et al., 2020, Complement Ther Clin Pract 39:101121</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>US Hispanic (nationally representative)</t>
+          <t>US; low-income, racially/ethnically diverse adults (~19% Hispanic/Latino); community-based</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Attitudinal familism measure showed factorial invariance across country of origin (US/Mexico/Latin America) and language (English/Spanish).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="118" customHeight="1">
+          <t>Significant pre/post improvements: sleep duration 5.4-&gt;6.9 h/night (p&lt;0.01), sleep-related impairment, sleep disturbance, and sleep-hygiene behaviors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="128" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/1073191111425856</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1389945726002583</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>The Brief Family Relationship Scale</t>
+          <t>Protocol for Nuestro Sueno: a randomized trial of a couples-based intervention to improve PAP adherence and sleep health among Hispanic patients beginning PAP and their partners</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Fok, Allen, Henry &amp; People Awakening Team, 2014, Assessment 21(1):67-72</t>
+          <t>2026, Sleep Medicine (protocol; NCT06649929; author byline not confirmed from snippets)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>US (Alaska Native youth; not Latino)</t>
+          <t>US + Latino; Hispanic couples; CHW-delivered telehealth</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Brief 16-item measure of the FES Relationship dimension (cohesion, expressiveness, conflict); validated as a family-functioning measure.</t>
+          <t>PROTOCOL ONLY - no outcomes yet. Pilot RCT testing a culturally adapted, community-health-worker-delivered couples intervention vs information control for PAP adherence and both partners' sleep.</t>
         </is>
       </c>
     </row>
@@ -1450,7 +1475,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>4. ICC Findings in Sleep Research</t>
+          <t>TAB 4 - Family cohesion measures</t>
         </is>
       </c>
     </row>
@@ -1481,165 +1506,165 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="118" customHeight="1">
+    <row r="3" ht="128" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/25845697/</t>
+          <t>https://doi.org/10.1111/j.1752-0606.2009.00175.x</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Reproducibility of a Standardized Actigraphy Scoring Algorithm for Sleep in a US Hispanic/Latino Population</t>
+          <t>FACES IV and the Circumplex Model: Validation Study</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Patel et al., 2015, Sleep 38(9):1497-1503</t>
+          <t>Olson, 2011, J Marital Fam Ther 37(1):64-80</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>US Hispanic/Latino (HCHS/SOL Sueno); 50 adults</t>
+          <t>US adults</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Reliability: intra- and inter-scorer ICCs 0.911-0.995 across all 11 actigraphy-derived sleep variables. Most directly relevant to US/Latino work.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="118" customHeight="1">
+          <t>Core validation of FACES IV; six scales span the cohesion continuum (balanced, disengaged, enmeshed) and flexibility, with strong concurrent, construct, and discriminant validity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="128" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/20191932/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/31853517/</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>A Twin Study of Sleep Duration and Body Mass Index</t>
+          <t>Measurement Properties of Sabogal's Familism Scale: Findings from the HCHS/SOL Sociocultural Ancillary Study</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Watson et al., 2010, J Clin Sleep Med 6(1):11-17</t>
+          <t>Campos et al., 2019, J Latinx Psychol 7(4):257-272 (DOI 10.1037/lat0000126)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>US adult twins</t>
+          <t>US Hispanic/Latino; N=5,313</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Family/genetic clustering: sleep-duration ICC ~2x larger in MZ than DZ twins -&gt; heritability 0.31 (p=0.08); BMI heritability 0.76.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="118" customHeight="1">
+          <t>Sabogal's 3-factor model (obligations, support, family as referents) fit well and was invariant across English/Spanish; good convergent/discriminant validity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="128" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s11325-025-03326-y</t>
+          <t>https://doi.org/10.1177/0739986303256912</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Moderately strong intraclass correlations between actigraphic and polysomnographic total sleep time and sleep efficiency in older adults with sleep disturbance</t>
+          <t>A New Familism Scale for Use with Latino Populations</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>2025, Sleep and Breathing 29(2):161 (CleverLights Study)</t>
+          <t>Lugo Steidel &amp; Contreras, 2003, Hisp J Behav Sci 25(3):312-330</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Older adults with sleep disturbance; n=12</t>
+          <t>US Latino adults; N=124</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Method agreement (actigraphy vs PSG): TST ICC 0.79; sleep efficiency 0.85; awakenings 0.45; TIB/WASO/SOL non-significant (0.30-0.33).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="118" customHeight="1">
+          <t>18-item scale, 4 factors (Support, Interconnectedness, Honor, Subjugation of Self), explaining ~51% of variance; overall alpha = .83.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="128" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/39833037/</t>
+          <t>https://doi.org/10.1177/0272431609338178</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Test-retest reliability of the Arabic version of the Pittsburgh Sleep Quality Index</t>
+          <t>The Mexican American Cultural Values Scale for Adolescents and Adults (MACVS)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Alqarni et al., 2025, Medicine (Baltimore) 104(3):e41269</t>
+          <t>Knight et al., 2010, J Early Adolesc 30(3):444-481</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Saudi Arabia (non-US); 202 students/interns</t>
+          <t>US Mexican American adolescents &amp; parents</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Questionnaire test-retest: overall PSQI ICC 0.694; sleep efficiency 0.460; sleep latency 0.730.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="118" customHeight="1">
+          <t>50-item, 9-subscale measure with three Familism subscales (Support, Referent, Obligation); supported the higher-order structure, reliability, and construct validity. English/Spanish.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="128" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1038/s41598-025-07786-w</t>
+          <t>https://doi.org/10.1177/0739986305281125</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Agreement between parental reports and accelerometer measures of sleep duration in primary school children</t>
+          <t>Factorial invariance of a pan-Hispanic familism scale</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Duarte, Martins &amp; Rosario, 2025, Scientific Reports</t>
+          <t>Villarreal, Blozis &amp; Widaman, 2005, Hisp J Behav Sci 27(4):409-425</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Portugal (non-US); 735 primary-school children</t>
+          <t>US Hispanic (nationally representative)</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Proxy-report agreement: weekday ICC 0.189, weekend 0.139 - poor parent-vs-accelerometer agreement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="118" customHeight="1">
+          <t>Attitudinal familism measure showed factorial invariance across country of origin (US/Mexico/Latin America) and language (English/Spanish).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="128" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/josh.13175</t>
+          <t>https://doi.org/10.1177/1073191111425856</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Effect Evaluation of a School-Based Intervention Promoting Sleep in Adolescents: A Cluster-Randomized Controlled Trial</t>
+          <t>The Brief Family Relationship Scale</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Inhulsen, Busch &amp; van Stralen, 2022, J School Health (PMID 35315076)</t>
+          <t>Fok, Allen, Henry &amp; People Awakening Team, 2014, Assessment 21(1):67-72</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Netherlands (non-US); 972 students, 10 high schools</t>
+          <t>US (Alaska Native youth; not Latino)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>DESIGN-ASSUMPTION benchmark (not empirically estimated): used an assumed school-level ICC of 0.10 for sleep duration in its cluster-RCT power calculation.</t>
+          <t>Brief 16-item measure of the FES Relationship dimension (cohesion, expressiveness, conflict); validated as a family-functioning measure.</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1690,235 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TAB 5 - Prior ICC findings in sleep research</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Paper link</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Authors / Year / Journal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Key relevant finding(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="128" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/25845697/</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Reproducibility of a Standardized Actigraphy Scoring Algorithm for Sleep in a US Hispanic/Latino Population</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Patel et al., 2015, Sleep 38(9):1497-1503</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>US Hispanic/Latino (HCHS/SOL Sueno); 50 adults</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Reliability: intra- and inter-scorer ICCs 0.911-0.995 across all 11 actigraphy-derived sleep variables. Most directly relevant to US/Latino work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="128" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/20191932/</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>A Twin Study of Sleep Duration and Body Mass Index</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Watson et al., 2010, J Clin Sleep Med 6(1):11-17</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>US adult twins</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Family/genetic clustering: sleep-duration ICC ~2x larger in MZ than DZ twins -&gt; heritability 0.31 (p=0.08); BMI heritability 0.76.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="128" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s11325-025-03326-y</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Moderately strong intraclass correlations between actigraphic and polysomnographic total sleep time and sleep efficiency in older adults with sleep disturbance</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2025, Sleep and Breathing 29(2):161 (CleverLights Study)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Older adults with sleep disturbance; n=12</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Method agreement (actigraphy vs PSG): TST ICC 0.79; sleep efficiency 0.85; awakenings 0.45; TIB/WASO/SOL non-significant (0.30-0.33).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="128" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/39833037/</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Test-retest reliability of the Arabic version of the Pittsburgh Sleep Quality Index</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Alqarni et al., 2025, Medicine (Baltimore) 104(3):e41269</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Saudi Arabia (non-US); 202 students/interns</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Questionnaire test-retest: overall PSQI ICC 0.694; sleep efficiency 0.460; sleep latency 0.730.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="128" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-025-07786-w</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Agreement between parental reports and accelerometer measures of sleep duration in primary school children</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Duarte, Martins &amp; Rosario, 2025, Scientific Reports</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Portugal (non-US); 735 primary-school children</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Proxy-report agreement: weekday ICC 0.189, weekend 0.139 - poor parent-vs-accelerometer agreement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="128" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/josh.13175</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Effect Evaluation of a School-Based Intervention Promoting Sleep in Adolescents: A Cluster-Randomized Controlled Trial</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Inhulsen, Busch &amp; van Stralen, 2022, J School Health (PMID 35315076)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Netherlands (non-US); 972 students, 10 high schools</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>DESIGN-ASSUMPTION benchmark (not empirically estimated): used an assumed school-level ICC of 0.10 for sleep duration in its cluster-RCT power calculation.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -1684,74 +1937,119 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>All 24 papers were verified: every DOI / PubMed ID / URL resolves to the stated article, and titles, authors, journals, and years match.</t>
+          <t>Tab 1 (Sleep Instruments) lists only VALIDATED, SCORED instruments that yield a computable household/family/sleep-environment score - the most useful for building a family/household sleep 'score'. Tab 2 collects family/household-level FACTORS shown to be associated with sleep (association studies, not scored instruments).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Peer-reviewed journal articles only. US and/or Latino/Hispanic populations prioritized; non-US or non-Latino items are foundational instruments/methods and are flagged in the Population column.</t>
+          <t>All papers were verified: DOIs / PubMed IDs / URLs resolve to the stated article, and titles/authors/journals/years match the published record.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr"/>
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Peer-reviewed journal articles only. US and/or Latino/Hispanic populations prioritized; non-US items are foundational instruments/methods and are flagged in the Population column.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Caveats:</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>- Community Interventions row 4 (Dominican Republic, Sleep Health 2016) and row 6 (Nuestro Sueno protocol, Sleep Medicine 2026): the articles definitely exist at the given URLs with confirmed titles, but author bylines could not be independently confirmed from search snippets. Verify authors on the publisher page.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>- Nuestro Sueno is a study PROTOCOL - it reports no outcome results yet.</t>
+          <t>- Tab 1, PSPQ (Meltzer 2021): author order taken from search-result/Tandfonline record (full text was proxy-blocked); title, journal, volume, year, DOI confirmed across sources.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>- ICC row 6 (Inhulsen 2022) reports an ASSUMED school-level ICC of 0.10 used in a power calculation, not an empirically estimated value.</t>
+          <t>- Tab 1, Household Crowding Index: the index (persons/room) is a long-standing construct; the two cited papers (Torshizian &amp; Grimes 2021; Cable &amp; Sacker 2019) are peer-reviewed validation/comparison studies used as the methodological basis.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr"/>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>- Tab 2, Housing crowding in urban China (Soc Sci Med 2025) and Tab 3, Dominican Republic (Sleep Health 2016) &amp; Nuestro Sueno (Sleep Medicine 2026): articles exist at the given URLs with confirmed titles, but author bylines could not be independently confirmed from snippets. Verify authors on the publisher page.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Literature gaps identified:</t>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>- Nuestro Sueno (Tab 3) is a study PROTOCOL - no outcome results yet.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>- No widely validated standalone 'family sleep health scale' beyond the FISH.</t>
+          <t>- ICC Tab, Inhulsen 2022 reports an ASSUMED school-level ICC of 0.10 used in a power calculation, not an empirically estimated value.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>- No completed, peer-reviewed promotora-delivered sleep intervention in US Latino adults with reported sleep outcomes yet (niche is at protocol/pilot stage).</t>
-        </is>
-      </c>
+      <c r="A13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Instruments considered but excluded from Tab 1 (do not meet 'scored household/family/environment' criterion):</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>- Sleep Hygiene Index (Mastin 2006): individual behaviors, no distinct scored environmental/household subscale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>- RU-SATED / composite sleep-health scores: individual-level, not family/household.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>- Children's Sleep Hygiene Scale (CSHS): has an environmental subscale but its primary citation is a conference abstract, not a full journal article; its content is captured by the CRSP (Tab 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Literature gaps:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>- No completed, peer-reviewed promotora-delivered sleep intervention in US Latino adults with reported sleep outcomes yet (niche at protocol/pilot stage).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>- Empirically estimated household- or clinic-level clustering ICCs for sleep are scarce; the twin heritability (0.31) and the assumed school-level ICC (0.10) are the closest anchors for multilevel design planning.</t>
         </is>

</xml_diff>

<commit_message>
Add Tab 1 Summary: scored instruments by population with proposal guidance
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017saKLUxckuv8JPxf8F2UXy
</commit_message>
<xml_diff>
--- a/sleep_literature_review.xlsx
+++ b/sleep_literature_review.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Sleep Instruments (scored)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Family Factors &amp; Sleep" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Community Interventions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Family Cohesion Measures" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ICC in Sleep Research" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Notes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Tab 1 Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Family Factors &amp; Sleep" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Community Interventions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Family Cohesion Measures" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ICC in Sleep Research" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Notes" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +49,19 @@
       <b val="1"/>
       <i val="1"/>
       <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
+    <font>
       <sz val="11"/>
     </font>
     <font>
@@ -98,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -112,17 +126,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -830,6 +853,295 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="118" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Tab 1 - Scored Sleep Instruments: summary for a family / household-level proposal</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Ten validated instruments that produce a numeric score/index. Grouped below by WHO reports and WHO the score is about, so a team can pick age-appropriate, multi-informant tools for a household.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>ADULTS - self-report</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>- ASE (Grandner 2022): scores the respondent's own bedroom/home sleep ENVIRONMENT (light, temperature, noise, safety, comfort, humidity, smell). Best single environment instrument; apply to each adult in the household.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>- SHPS (Yang 2010): scores adult sleep-hygiene PRACTICES, including a dedicated sleep-environment domain. Broader than ASE (also schedule, arousal, eating/drinking).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>ADOLESCENTS - self-report</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>- ASHS-r (Storfer-Isser 2013): adolescent (~16-19 yr) sleep-hygiene score with a scored sleep-ENVIRONMENT subscale (plus physiological, arousal, cognitive/emotional, daytime sleep, stability).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>SCHOOL-AGE CHILDREN / YOUTH - child self-report</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>- CRSP (Meltzer 2013): children 8-12 self-report; the Sleep Hygiene module has a scored ENVIRONMENTAL subscale. Lets the child (not just the parent) rate their environment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>- PSPQ (Meltzer 2021): youth 8-17 self-report; scores 5 sleep practices including a room-ENVIRONMENT subscale, plus timing, routines, technology use, parental presence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>CHILDREN - caregiver / parent-report</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>- FISH (Malow 2009): the ONLY true FAMILY-UNIT score here - parent-reported family sleep hygiene covering routines, sleep environment, AND parental bedtime behaviors (children ~4-10 yr). Natural anchor for a family-level design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>- CASES (Peltz 2022): caregiver-report score of the child's sleep ENVIRONMENT (hazards, bedding availability, electronics) for children 5-18 yr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>- BRQ (Henderson &amp; Jordan 2010): caregiver-report score of children's BEDTIME ROUTINES (children 2-8 yr; reactive vs. consistent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>INFANTS / NEWBORNS - caregiver-report</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>- Parent Newborn Sleep Safety Survey (Whiteside-Mansell 2017): scores caregiver adherence to safe-sleep-ENVIRONMENT recommendations (position, surface, bedding, location). Validated against direct observation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>WHOLE HOUSEHOLD - objective / computed (no self-report)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>- Household Crowding Index (Torshizian &amp; Grimes 2021; Cable &amp; Sacker 2019): a computed persons-per-room index. An objective structural covariate for the household - ideal for adjustment/multilevel models, not reliant on perception.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>WHAT EACH SCORES (quick construct map)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>- Physical sleep environment (core): ASE, CASES; environment SUBSCALES within ASHS-r, SHPS, CRSP, PSPQ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>- Broader sleep hygiene / practices: SHPS, ASHS-r, CRSP, PSPQ, FISH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>- Bedtime routines: BRQ, FISH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>- Safe-sleep environment (infants): Parent Newborn Sleep Safety Survey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>- Objective household structure: Household Crowding Index.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>PRACTICAL GUIDANCE FOR A FAMILY / HOUSEHOLD INTERVENTION OR DATA COLLECTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>- Anchor on FISH for a genuine family-level score - it is the only instrument that scores the family unit (including parental bedtime behaviors), not just one individual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>- Go multi-informant within a household: pair a caregiver-report (FISH / CASES / BRQ) with a child or adolescent self-report (CRSP / PSPQ / ASHS-r) so child and parent both rate the same home.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>- Add ASE for each adult to capture the physical bedroom environment directly; it is the most focused, well-validated environment score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>- Include the Household Crowding Index as an objective, low-burden covariate that does not depend on self-report - useful for confounding adjustment and multilevel (household-clustered) models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>- Cover the household lifespan by choosing age-appropriate tools: infant (Newborn Safety Survey) -&gt; toddler/preschool (BRQ 2-8, FISH 4-10) -&gt; school-age (CRSP 8-12, CASES 5-18, PSPQ 8-17) -&gt; adolescent (ASHS-r ~16-19) -&gt; adult (ASE, SHPS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>- If the intervention TARGET is the physical/home environment, prioritize ASE + CASES (+ Crowding Index); if the target is routines/behaviors, prioritize FISH + BRQ (+ PSPQ/CRSP for the child's view).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>CAVEATS / GAPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>- Most environment instruments were validated in US samples; SHPS is Taiwanese. Confirm cross-cultural/Spanish-language validity before use in Latino samples (a documented gap - see Blanco 2024 in Tab 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>- Only FISH scores the family as a unit; the others score an individual or the physical/structural environment. A single 'validated whole-family household sleep score' does not yet exist - a family-level composite would likely combine several of these.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>- PSPQ author order and the Crowding Index details carry the verification caveats noted in the Notes sheet.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -875,15 +1187,15 @@
       </c>
     </row>
     <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Family routines, parenting &amp; sociodemographics</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
+      <c r="B3" s="11" t="n"/>
+      <c r="C3" s="11" t="n"/>
+      <c r="D3" s="11" t="n"/>
+      <c r="E3" s="11" t="n"/>
     </row>
     <row r="4" ht="128" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -967,15 +1279,15 @@
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Household crowding &amp; room/bed sharing</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
     </row>
     <row r="8" ht="128" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -1059,15 +1371,15 @@
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Housing type / quality &amp; neighborhood physical environment</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
     </row>
     <row r="12" ht="128" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -1228,234 +1540,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>TAB 3 - Community sleep interventions</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Paper link</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Authors / Year / Journal</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Key relevant finding(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="128" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1177/00099228231207307</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>A Pilot Randomized Control Trial Demonstrating the Efficacy of the SIESTA Sleep Hygiene Intervention</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Koinis-Mitchell et al., 2024, Clinical Pediatrics 63(8):1062-1077</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>US + Latino; urban Latino middle-schoolers (Providence RI &amp; San Juan PR); school-based, bilingual</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Actigraphy sleep duration rose 13.3% (~45 min) in SIESTA vs 7.2% (~25 min) in controls; child- and caregiver-reported sleep disturbances significantly decreased through 4-month follow-up.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="128" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.5664/jcsm.8510</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Tailored Approach to Sleep Health Education (TASHE): a randomized controlled trial of a web-based application</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Jean-Louis et al., 2020, J Clin Sleep Med 16(8):1331-1341</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>US, Black; 194 adults at high OSA risk; community-engaged (barbershops, salons, places of worship)</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>TASHE group showed increased sleep hygiene over 6 months vs control; no significant change in OSA beliefs or knowledge.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="128" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1111/jsr.14213</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Effectiveness of peer-delivered sleep health education and social support in increasing OSA evaluation among at-risk blacks</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Jean-Louis et al., 2025, J Sleep Res 34(1):e14213</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>US, Black; 319 adults at OSA risk; peer/community-delivered</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Peer-based social support and psychosocial factors favorably related to OSA evaluation/adherence behavior vs standard information.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="128" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sciencedirect.com/science/article/abs/pii/S2352721816000188</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Efficacy of sleep education in a Dominican Republic neighborhood through training of community health promoters</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>2016, Sleep Health (author byline not confirmed from snippets)</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Dominican Republic (Latino, non-US); community members + 9 health promoters</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Promoters' sleep-disorder knowledge improved after a 4-hr training, but community members' knowledge did not significantly change after promoter-delivered education.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="128" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.ctcp.2020.101121</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>A sleep hygiene and yoga intervention conducted in affordable housing communities: pilot study results and lessons for a future trial</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Spadola et al., 2020, Complement Ther Clin Pract 39:101121</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>US; low-income, racially/ethnically diverse adults (~19% Hispanic/Latino); community-based</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Significant pre/post improvements: sleep duration 5.4-&gt;6.9 h/night (p&lt;0.01), sleep-related impairment, sleep disturbance, and sleep-hygiene behaviors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="128" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S1389945726002583</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Protocol for Nuestro Sueno: a randomized trial of a couples-based intervention to improve PAP adherence and sleep health among Hispanic patients beginning PAP and their partners</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>2026, Sleep Medicine (protocol; NCT06649929; author byline not confirmed from snippets)</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>US + Latino; Hispanic couples; CHW-delivered telehealth</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>PROTOCOL ONLY - no outcomes yet. Pilot RCT testing a culturally adapted, community-health-worker-delivered couples intervention vs information control for PAP adherence and both partners' sleep.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId6"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1475,7 +1559,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TAB 4 - Family cohesion measures</t>
+          <t>TAB 3 - Community sleep interventions</t>
         </is>
       </c>
     </row>
@@ -1509,162 +1593,162 @@
     <row r="3" ht="128" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/j.1752-0606.2009.00175.x</t>
+          <t>https://doi.org/10.1177/00099228231207307</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>FACES IV and the Circumplex Model: Validation Study</t>
+          <t>A Pilot Randomized Control Trial Demonstrating the Efficacy of the SIESTA Sleep Hygiene Intervention</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Olson, 2011, J Marital Fam Ther 37(1):64-80</t>
+          <t>Koinis-Mitchell et al., 2024, Clinical Pediatrics 63(8):1062-1077</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>US adults</t>
+          <t>US + Latino; urban Latino middle-schoolers (Providence RI &amp; San Juan PR); school-based, bilingual</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Core validation of FACES IV; six scales span the cohesion continuum (balanced, disengaged, enmeshed) and flexibility, with strong concurrent, construct, and discriminant validity.</t>
+          <t>Actigraphy sleep duration rose 13.3% (~45 min) in SIESTA vs 7.2% (~25 min) in controls; child- and caregiver-reported sleep disturbances significantly decreased through 4-month follow-up.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="128" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/31853517/</t>
+          <t>https://doi.org/10.5664/jcsm.8510</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Measurement Properties of Sabogal's Familism Scale: Findings from the HCHS/SOL Sociocultural Ancillary Study</t>
+          <t>Tailored Approach to Sleep Health Education (TASHE): a randomized controlled trial of a web-based application</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Campos et al., 2019, J Latinx Psychol 7(4):257-272 (DOI 10.1037/lat0000126)</t>
+          <t>Jean-Louis et al., 2020, J Clin Sleep Med 16(8):1331-1341</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>US Hispanic/Latino; N=5,313</t>
+          <t>US, Black; 194 adults at high OSA risk; community-engaged (barbershops, salons, places of worship)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Sabogal's 3-factor model (obligations, support, family as referents) fit well and was invariant across English/Spanish; good convergent/discriminant validity.</t>
+          <t>TASHE group showed increased sleep hygiene over 6 months vs control; no significant change in OSA beliefs or knowledge.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="128" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/0739986303256912</t>
+          <t>https://doi.org/10.1111/jsr.14213</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>A New Familism Scale for Use with Latino Populations</t>
+          <t>Effectiveness of peer-delivered sleep health education and social support in increasing OSA evaluation among at-risk blacks</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Lugo Steidel &amp; Contreras, 2003, Hisp J Behav Sci 25(3):312-330</t>
+          <t>Jean-Louis et al., 2025, J Sleep Res 34(1):e14213</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>US Latino adults; N=124</t>
+          <t>US, Black; 319 adults at OSA risk; peer/community-delivered</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>18-item scale, 4 factors (Support, Interconnectedness, Honor, Subjugation of Self), explaining ~51% of variance; overall alpha = .83.</t>
+          <t>Peer-based social support and psychosocial factors favorably related to OSA evaluation/adherence behavior vs standard information.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="128" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/0272431609338178</t>
+          <t>https://www.sciencedirect.com/science/article/abs/pii/S2352721816000188</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>The Mexican American Cultural Values Scale for Adolescents and Adults (MACVS)</t>
+          <t>Efficacy of sleep education in a Dominican Republic neighborhood through training of community health promoters</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Knight et al., 2010, J Early Adolesc 30(3):444-481</t>
+          <t>2016, Sleep Health (author byline not confirmed from snippets)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>US Mexican American adolescents &amp; parents</t>
+          <t>Dominican Republic (Latino, non-US); community members + 9 health promoters</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>50-item, 9-subscale measure with three Familism subscales (Support, Referent, Obligation); supported the higher-order structure, reliability, and construct validity. English/Spanish.</t>
+          <t>Promoters' sleep-disorder knowledge improved after a 4-hr training, but community members' knowledge did not significantly change after promoter-delivered education.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="128" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/0739986305281125</t>
+          <t>https://doi.org/10.1016/j.ctcp.2020.101121</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Factorial invariance of a pan-Hispanic familism scale</t>
+          <t>A sleep hygiene and yoga intervention conducted in affordable housing communities: pilot study results and lessons for a future trial</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Villarreal, Blozis &amp; Widaman, 2005, Hisp J Behav Sci 27(4):409-425</t>
+          <t>Spadola et al., 2020, Complement Ther Clin Pract 39:101121</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>US Hispanic (nationally representative)</t>
+          <t>US; low-income, racially/ethnically diverse adults (~19% Hispanic/Latino); community-based</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Attitudinal familism measure showed factorial invariance across country of origin (US/Mexico/Latin America) and language (English/Spanish).</t>
+          <t>Significant pre/post improvements: sleep duration 5.4-&gt;6.9 h/night (p&lt;0.01), sleep-related impairment, sleep disturbance, and sleep-hygiene behaviors.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="128" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/1073191111425856</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1389945726002583</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>The Brief Family Relationship Scale</t>
+          <t>Protocol for Nuestro Sueno: a randomized trial of a couples-based intervention to improve PAP adherence and sleep health among Hispanic patients beginning PAP and their partners</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Fok, Allen, Henry &amp; People Awakening Team, 2014, Assessment 21(1):67-72</t>
+          <t>2026, Sleep Medicine (protocol; NCT06649929; author byline not confirmed from snippets)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>US (Alaska Native youth; not Latino)</t>
+          <t>US + Latino; Hispanic couples; CHW-delivered telehealth</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Brief 16-item measure of the FES Relationship dimension (cohesion, expressiveness, conflict); validated as a family-functioning measure.</t>
+          <t>PROTOCOL ONLY - no outcomes yet. Pilot RCT testing a culturally adapted, community-health-worker-delivered couples intervention vs information control for PAP adherence and both partners' sleep.</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1787,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TAB 5 - Prior ICC findings in sleep research</t>
+          <t>TAB 4 - Family cohesion measures</t>
         </is>
       </c>
     </row>
@@ -1737,162 +1821,162 @@
     <row r="3" ht="128" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/25845697/</t>
+          <t>https://doi.org/10.1111/j.1752-0606.2009.00175.x</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Reproducibility of a Standardized Actigraphy Scoring Algorithm for Sleep in a US Hispanic/Latino Population</t>
+          <t>FACES IV and the Circumplex Model: Validation Study</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Patel et al., 2015, Sleep 38(9):1497-1503</t>
+          <t>Olson, 2011, J Marital Fam Ther 37(1):64-80</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>US Hispanic/Latino (HCHS/SOL Sueno); 50 adults</t>
+          <t>US adults</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Reliability: intra- and inter-scorer ICCs 0.911-0.995 across all 11 actigraphy-derived sleep variables. Most directly relevant to US/Latino work.</t>
+          <t>Core validation of FACES IV; six scales span the cohesion continuum (balanced, disengaged, enmeshed) and flexibility, with strong concurrent, construct, and discriminant validity.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="128" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/20191932/</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/31853517/</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>A Twin Study of Sleep Duration and Body Mass Index</t>
+          <t>Measurement Properties of Sabogal's Familism Scale: Findings from the HCHS/SOL Sociocultural Ancillary Study</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Watson et al., 2010, J Clin Sleep Med 6(1):11-17</t>
+          <t>Campos et al., 2019, J Latinx Psychol 7(4):257-272 (DOI 10.1037/lat0000126)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>US adult twins</t>
+          <t>US Hispanic/Latino; N=5,313</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Family/genetic clustering: sleep-duration ICC ~2x larger in MZ than DZ twins -&gt; heritability 0.31 (p=0.08); BMI heritability 0.76.</t>
+          <t>Sabogal's 3-factor model (obligations, support, family as referents) fit well and was invariant across English/Spanish; good convergent/discriminant validity.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="128" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s11325-025-03326-y</t>
+          <t>https://doi.org/10.1177/0739986303256912</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Moderately strong intraclass correlations between actigraphic and polysomnographic total sleep time and sleep efficiency in older adults with sleep disturbance</t>
+          <t>A New Familism Scale for Use with Latino Populations</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>2025, Sleep and Breathing 29(2):161 (CleverLights Study)</t>
+          <t>Lugo Steidel &amp; Contreras, 2003, Hisp J Behav Sci 25(3):312-330</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Older adults with sleep disturbance; n=12</t>
+          <t>US Latino adults; N=124</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Method agreement (actigraphy vs PSG): TST ICC 0.79; sleep efficiency 0.85; awakenings 0.45; TIB/WASO/SOL non-significant (0.30-0.33).</t>
+          <t>18-item scale, 4 factors (Support, Interconnectedness, Honor, Subjugation of Self), explaining ~51% of variance; overall alpha = .83.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="128" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>https://pubmed.ncbi.nlm.nih.gov/39833037/</t>
+          <t>https://doi.org/10.1177/0272431609338178</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Test-retest reliability of the Arabic version of the Pittsburgh Sleep Quality Index</t>
+          <t>The Mexican American Cultural Values Scale for Adolescents and Adults (MACVS)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Alqarni et al., 2025, Medicine (Baltimore) 104(3):e41269</t>
+          <t>Knight et al., 2010, J Early Adolesc 30(3):444-481</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Saudi Arabia (non-US); 202 students/interns</t>
+          <t>US Mexican American adolescents &amp; parents</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Questionnaire test-retest: overall PSQI ICC 0.694; sleep efficiency 0.460; sleep latency 0.730.</t>
+          <t>50-item, 9-subscale measure with three Familism subscales (Support, Referent, Obligation); supported the higher-order structure, reliability, and construct validity. English/Spanish.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="128" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1038/s41598-025-07786-w</t>
+          <t>https://doi.org/10.1177/0739986305281125</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Agreement between parental reports and accelerometer measures of sleep duration in primary school children</t>
+          <t>Factorial invariance of a pan-Hispanic familism scale</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Duarte, Martins &amp; Rosario, 2025, Scientific Reports</t>
+          <t>Villarreal, Blozis &amp; Widaman, 2005, Hisp J Behav Sci 27(4):409-425</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Portugal (non-US); 735 primary-school children</t>
+          <t>US Hispanic (nationally representative)</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Proxy-report agreement: weekday ICC 0.189, weekend 0.139 - poor parent-vs-accelerometer agreement.</t>
+          <t>Attitudinal familism measure showed factorial invariance across country of origin (US/Mexico/Latin America) and language (English/Spanish).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="128" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/josh.13175</t>
+          <t>https://doi.org/10.1177/1073191111425856</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Effect Evaluation of a School-Based Intervention Promoting Sleep in Adolescents: A Cluster-Randomized Controlled Trial</t>
+          <t>The Brief Family Relationship Scale</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Inhulsen, Busch &amp; van Stralen, 2022, J School Health (PMID 35315076)</t>
+          <t>Fok, Allen, Henry &amp; People Awakening Team, 2014, Assessment 21(1):67-72</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Netherlands (non-US); 972 students, 10 high schools</t>
+          <t>US (Alaska Native youth; not Latino)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>DESIGN-ASSUMPTION benchmark (not empirically estimated): used an assumed school-level ICC of 0.10 for sleep duration in its cluster-RCT power calculation.</t>
+          <t>Brief 16-item measure of the FES Relationship dimension (cohesion, expressiveness, conflict); validated as a family-functioning measure.</t>
         </is>
       </c>
     </row>
@@ -1918,6 +2002,234 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TAB 5 - Prior ICC findings in sleep research</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Paper link</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Authors / Year / Journal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Key relevant finding(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="128" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/25845697/</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Reproducibility of a Standardized Actigraphy Scoring Algorithm for Sleep in a US Hispanic/Latino Population</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Patel et al., 2015, Sleep 38(9):1497-1503</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>US Hispanic/Latino (HCHS/SOL Sueno); 50 adults</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Reliability: intra- and inter-scorer ICCs 0.911-0.995 across all 11 actigraphy-derived sleep variables. Most directly relevant to US/Latino work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="128" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/20191932/</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>A Twin Study of Sleep Duration and Body Mass Index</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Watson et al., 2010, J Clin Sleep Med 6(1):11-17</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>US adult twins</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Family/genetic clustering: sleep-duration ICC ~2x larger in MZ than DZ twins -&gt; heritability 0.31 (p=0.08); BMI heritability 0.76.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="128" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s11325-025-03326-y</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Moderately strong intraclass correlations between actigraphic and polysomnographic total sleep time and sleep efficiency in older adults with sleep disturbance</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2025, Sleep and Breathing 29(2):161 (CleverLights Study)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Older adults with sleep disturbance; n=12</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Method agreement (actigraphy vs PSG): TST ICC 0.79; sleep efficiency 0.85; awakenings 0.45; TIB/WASO/SOL non-significant (0.30-0.33).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="128" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>https://pubmed.ncbi.nlm.nih.gov/39833037/</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Test-retest reliability of the Arabic version of the Pittsburgh Sleep Quality Index</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Alqarni et al., 2025, Medicine (Baltimore) 104(3):e41269</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Saudi Arabia (non-US); 202 students/interns</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Questionnaire test-retest: overall PSQI ICC 0.694; sleep efficiency 0.460; sleep latency 0.730.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="128" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-025-07786-w</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Agreement between parental reports and accelerometer measures of sleep duration in primary school children</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Duarte, Martins &amp; Rosario, 2025, Scientific Reports</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Portugal (non-US); 735 primary-school children</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Proxy-report agreement: weekday ICC 0.189, weekend 0.139 - poor parent-vs-accelerometer agreement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="128" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/josh.13175</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Effect Evaluation of a School-Based Intervention Promoting Sleep in Adolescents: A Cluster-Randomized Controlled Trial</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Inhulsen, Busch &amp; van Stralen, 2022, J School Health (PMID 35315076)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Netherlands (non-US); 972 students, 10 high schools</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>DESIGN-ASSUMPTION benchmark (not empirically estimated): used an assumed school-level ICC of 0.10 for sleep duration in its cluster-RCT power calculation.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1925,131 +2237,131 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Verification &amp; scope notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr"/>
+      <c r="A2" s="7" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Tab 1 (Sleep Instruments) lists only VALIDATED, SCORED instruments that yield a computable household/family/sleep-environment score - the most useful for building a family/household sleep 'score'. Tab 2 collects family/household-level FACTORS shown to be associated with sleep (association studies, not scored instruments).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>All papers were verified: DOIs / PubMed IDs / URLs resolve to the stated article, and titles/authors/journals/years match the published record.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Peer-reviewed journal articles only. US and/or Latino/Hispanic populations prioritized; non-US items are foundational instruments/methods and are flagged in the Population column.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr"/>
+      <c r="A6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Caveats:</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>- Tab 1, PSPQ (Meltzer 2021): author order taken from search-result/Tandfonline record (full text was proxy-blocked); title, journal, volume, year, DOI confirmed across sources.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>- Tab 1, Household Crowding Index: the index (persons/room) is a long-standing construct; the two cited papers (Torshizian &amp; Grimes 2021; Cable &amp; Sacker 2019) are peer-reviewed validation/comparison studies used as the methodological basis.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>- Tab 2, Housing crowding in urban China (Soc Sci Med 2025) and Tab 3, Dominican Republic (Sleep Health 2016) &amp; Nuestro Sueno (Sleep Medicine 2026): articles exist at the given URLs with confirmed titles, but author bylines could not be independently confirmed from snippets. Verify authors on the publisher page.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>- Nuestro Sueno (Tab 3) is a study PROTOCOL - no outcome results yet.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>- ICC Tab, Inhulsen 2022 reports an ASSUMED school-level ICC of 0.10 used in a power calculation, not an empirically estimated value.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr"/>
+      <c r="A13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Instruments considered but excluded from Tab 1 (do not meet 'scored household/family/environment' criterion):</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>- Sleep Hygiene Index (Mastin 2006): individual behaviors, no distinct scored environmental/household subscale.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>- RU-SATED / composite sleep-health scores: individual-level, not family/household.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>- Children's Sleep Hygiene Scale (CSHS): has an environmental subscale but its primary citation is a conference abstract, not a full journal article; its content is captured by the CRSP (Tab 1).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr"/>
+      <c r="A18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Literature gaps:</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>- No completed, peer-reviewed promotora-delivered sleep intervention in US Latino adults with reported sleep outcomes yet (niche at protocol/pilot stage).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>- Empirically estimated household- or clinic-level clustering ICCs for sleep are scarce; the twin heritability (0.31) and the assumed school-level ICC (0.10) are the closest anchors for multilevel design planning.</t>
         </is>

</xml_diff>